<commit_message>
set up files for excel example and fix google drive function and update readme
</commit_message>
<xml_diff>
--- a/resources/read_excel_workbook_examples/data_excel/ClinicA.xlsx
+++ b/resources/read_excel_workbook_examples/data_excel/ClinicA.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GIT\DairyHealthDataProcessing\resources\read_excel_workbook_examples\data_excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{090D2384-4959-4D31-8464-87274322C41F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{48BD1CE6-E3BF-4EE6-B9EB-FF4F29CBFF62}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" activeTab="1" xr2:uid="{98C36F96-D751-4246-A510-4151DE36194D}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{98C36F96-D751-4246-A510-4151DE36194D}"/>
   </bookViews>
   <sheets>
     <sheet name="H1" sheetId="1" r:id="rId1"/>
@@ -70,6 +70,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="165" formatCode="yyyy\-mm\-dd;@"/>
+  </numFmts>
   <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -105,9 +108,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="16" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -620,6 +624,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EBF839E9-8416-4C1A-B4D3-5B3A865BC7B7}">
   <dimension ref="A1:C23"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <cols>
+    <col min="3" max="3" width="9.9296875" style="2" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A1" t="s">
@@ -628,7 +635,7 @@
       <c r="B1" t="s">
         <v>0</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="2" t="s">
         <v>1</v>
       </c>
     </row>
@@ -639,7 +646,7 @@
       <c r="B2" t="s">
         <v>3</v>
       </c>
-      <c r="C2" s="1">
+      <c r="C2" s="2">
         <v>46023</v>
       </c>
     </row>
@@ -650,7 +657,7 @@
       <c r="B3" t="s">
         <v>3</v>
       </c>
-      <c r="C3" s="1">
+      <c r="C3" s="2">
         <v>46024</v>
       </c>
     </row>
@@ -661,7 +668,7 @@
       <c r="B4" t="s">
         <v>4</v>
       </c>
-      <c r="C4" s="1">
+      <c r="C4" s="2">
         <v>46025</v>
       </c>
     </row>
@@ -672,7 +679,7 @@
       <c r="B5" t="s">
         <v>5</v>
       </c>
-      <c r="C5" s="1">
+      <c r="C5" s="2">
         <v>46026</v>
       </c>
     </row>
@@ -683,7 +690,7 @@
       <c r="B6" t="s">
         <v>3</v>
       </c>
-      <c r="C6" s="1">
+      <c r="C6" s="2">
         <v>46027</v>
       </c>
     </row>
@@ -694,7 +701,7 @@
       <c r="B7" t="s">
         <v>3</v>
       </c>
-      <c r="C7" s="1">
+      <c r="C7" s="2">
         <v>46028</v>
       </c>
     </row>
@@ -705,7 +712,7 @@
       <c r="B8" t="s">
         <v>3</v>
       </c>
-      <c r="C8" s="1">
+      <c r="C8" s="2">
         <v>46029</v>
       </c>
     </row>
@@ -716,7 +723,7 @@
       <c r="B9" t="s">
         <v>6</v>
       </c>
-      <c r="C9" s="1">
+      <c r="C9" s="2">
         <v>46030</v>
       </c>
     </row>
@@ -727,7 +734,7 @@
       <c r="B10" t="s">
         <v>3</v>
       </c>
-      <c r="C10" s="1">
+      <c r="C10" s="2">
         <v>46031</v>
       </c>
     </row>
@@ -738,7 +745,7 @@
       <c r="B11" t="s">
         <v>3</v>
       </c>
-      <c r="C11" s="1">
+      <c r="C11" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -749,7 +756,7 @@
       <c r="B12" t="s">
         <v>3</v>
       </c>
-      <c r="C12" s="1">
+      <c r="C12" s="2">
         <v>46033</v>
       </c>
     </row>
@@ -760,7 +767,7 @@
       <c r="B13" t="s">
         <v>5</v>
       </c>
-      <c r="C13" s="1">
+      <c r="C13" s="2">
         <v>46034</v>
       </c>
     </row>
@@ -771,7 +778,7 @@
       <c r="B14" t="s">
         <v>5</v>
       </c>
-      <c r="C14" s="1">
+      <c r="C14" s="2">
         <v>46035</v>
       </c>
     </row>
@@ -782,7 +789,7 @@
       <c r="B15" t="s">
         <v>5</v>
       </c>
-      <c r="C15" s="1">
+      <c r="C15" s="2">
         <v>46036</v>
       </c>
     </row>
@@ -793,7 +800,7 @@
       <c r="B16" t="s">
         <v>7</v>
       </c>
-      <c r="C16" s="1">
+      <c r="C16" s="2">
         <v>46037</v>
       </c>
     </row>
@@ -804,7 +811,7 @@
       <c r="B17" t="s">
         <v>7</v>
       </c>
-      <c r="C17" s="1">
+      <c r="C17" s="2">
         <v>46038</v>
       </c>
     </row>
@@ -815,7 +822,7 @@
       <c r="B18" t="s">
         <v>7</v>
       </c>
-      <c r="C18" s="1">
+      <c r="C18" s="2">
         <v>46039</v>
       </c>
     </row>
@@ -826,7 +833,7 @@
       <c r="B19" t="s">
         <v>7</v>
       </c>
-      <c r="C19" s="1">
+      <c r="C19" s="2">
         <v>46040</v>
       </c>
     </row>
@@ -837,7 +844,7 @@
       <c r="B20" t="s">
         <v>7</v>
       </c>
-      <c r="C20" s="1">
+      <c r="C20" s="2">
         <v>46041</v>
       </c>
     </row>
@@ -848,7 +855,7 @@
       <c r="B21" t="s">
         <v>7</v>
       </c>
-      <c r="C21" s="1">
+      <c r="C21" s="2">
         <v>46042</v>
       </c>
     </row>
@@ -859,7 +866,7 @@
       <c r="B22" t="s">
         <v>7</v>
       </c>
-      <c r="C22" s="1">
+      <c r="C22" s="2">
         <v>46043</v>
       </c>
     </row>
@@ -870,7 +877,7 @@
       <c r="B23" t="s">
         <v>7</v>
       </c>
-      <c r="C23" s="1">
+      <c r="C23" s="2">
         <v>46044</v>
       </c>
     </row>

</xml_diff>